<commit_message>
Name archived workbook sheets and refresh provenance checksums
</commit_message>
<xml_diff>
--- a/data/research_lifecycle_benchmark_100_msr27.xlsx
+++ b/data/research_lifecycle_benchmark_100_msr27.xlsx
@@ -7,12 +7,12 @@
     <sheet state="visible" name="reviewer2" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="agreement" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="final_agreement" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Hoja 11" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Hoja 12" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="Hoja 13" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="Hoja 14" sheetId="8" r:id="rId12"/>
-    <sheet state="visible" name="Hoja 15" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="Hoja 16" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="chatgpt_documentation" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="chatgpt_code" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="chatgpt_combined" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="heuristics_documentation" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="heuristics_code" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="heuristics_combined" sheetId="10" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="3" name="Z_892DE2D8_4F92_4535_843B_1DB18D037039_.wvu.FilterData">final_agreement!$A$1:$G$101</definedName>

</xml_diff>